<commit_message>
Added Centre of Gravity Calculation to conceptual_weights.mlx, amended table headers of mass_input.xlsx to aid in this
</commit_message>
<xml_diff>
--- a/HER04/mass_input.xlsx
+++ b/HER04/mass_input.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ash\Documents\University Files\Year 3\GDP\gdp_repo\HER04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCEFFA48-166B-4FFF-B0BF-FE2B7635D844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D396D829-044D-4E39-AD53-1075F91A1F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,21 +25,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Component</t>
   </si>
   <si>
-    <t>Mass/kg</t>
-  </si>
-  <si>
-    <t>x/m</t>
-  </si>
-  <si>
-    <t>y/m</t>
-  </si>
-  <si>
-    <t>z/m</t>
+    <t>test1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test2 </t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>z</t>
   </si>
 </sst>
 </file>
@@ -357,7 +363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
@@ -368,16 +374,50 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
+      <c r="B3">
+        <v>300</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added calculation of moments of inertia, updated files to match
</commit_message>
<xml_diff>
--- a/HER04/mass_input.xlsx
+++ b/HER04/mass_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ash\Documents\University Files\Year 3\GDP\gdp_repo\HER04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D396D829-044D-4E39-AD53-1075F91A1F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE821BA1-187A-4125-9C76-BE6E5322F19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Component</t>
   </si>
@@ -46,6 +46,24 @@
   </si>
   <si>
     <t>z</t>
+  </si>
+  <si>
+    <t>i_xx</t>
+  </si>
+  <si>
+    <t>i_yy</t>
+  </si>
+  <si>
+    <t>i_zz</t>
+  </si>
+  <si>
+    <t>i_xy</t>
+  </si>
+  <si>
+    <t>i_xz</t>
+  </si>
+  <si>
+    <t>i_zy</t>
   </si>
 </sst>
 </file>
@@ -363,13 +381,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -385,8 +403,26 @@
       <c r="E1" t="s">
         <v>6</v>
       </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -402,8 +438,26 @@
       <c r="E2">
         <v>1</v>
       </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -418,6 +472,24 @@
       </c>
       <c r="E3">
         <v>1</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed test line items from mass_input.xlsx
</commit_message>
<xml_diff>
--- a/HER04/mass_input.xlsx
+++ b/HER04/mass_input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/clarabollengandolfo/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ash\Documents\University Files\Year 3\GDP\gdp_repo\HER04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF175767-FCE1-2147-8E62-B7A09302A3C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFD2EEC-2BF1-4876-BDE4-CF8DE03E7E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
@@ -25,15 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Component</t>
-  </si>
-  <si>
-    <t>test1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test2 </t>
   </si>
   <si>
     <t>m</t>
@@ -408,140 +402,121 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" t="s">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="K1" t="s">
+      <c r="B2">
+        <v>47</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>2.1</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>100</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="B3">
+        <v>40</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>5.3</v>
+      </c>
+      <c r="E3">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4">
+        <v>256</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>5.3</v>
+      </c>
+      <c r="E4">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>300</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
-        <v>2.1</v>
+        <v>5.3</v>
       </c>
       <c r="E5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6">
-        <v>40</v>
+        <v>275</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -550,15 +525,15 @@
         <v>5.3</v>
       </c>
       <c r="E6">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
       <c r="B7">
-        <v>256</v>
+        <v>50</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -567,15 +542,15 @@
         <v>5.3</v>
       </c>
       <c r="E7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8">
-        <v>50</v>
+        <v>275</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -584,91 +559,40 @@
         <v>5.3</v>
       </c>
       <c r="E8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>18</v>
       </c>
       <c r="B9">
-        <v>275</v>
+        <v>100</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
       <c r="D9">
-        <v>5.3</v>
+        <v>10.3</v>
       </c>
       <c r="E9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B10">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
       <c r="D10">
-        <v>5.3</v>
+        <v>12.58</v>
       </c>
       <c r="E10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11">
-        <v>275</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>5.3</v>
-      </c>
-      <c r="E11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12">
-        <v>100</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>10.3</v>
-      </c>
-      <c r="E12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13">
-        <v>66</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>12.58</v>
-      </c>
-      <c r="E13">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
correction to mistake in mass_input.xlsx
</commit_message>
<xml_diff>
--- a/HER04/mass_input.xlsx
+++ b/HER04/mass_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ash\Documents\University Files\Year 3\GDP\gdp_repo\HER04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFD2EEC-2BF1-4876-BDE4-CF8DE03E7E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50428035-926B-413C-8176-94F3741D0CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -590,7 +590,7 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>12.58</v>
+        <v>12.8</v>
       </c>
       <c r="E10">
         <v>2</v>

</xml_diff>

<commit_message>
Updated positions and masses, now should have CG estimate
</commit_message>
<xml_diff>
--- a/HER04/mass_input.xlsx
+++ b/HER04/mass_input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ash\Documents\University Files\Year 3\GDP\gdp_repo\HER04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{728CB064-2882-4617-BAAA-D766DDB68A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4BD704-E5C9-47D3-A534-740327A794C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Component</t>
   </si>
@@ -71,36 +71,9 @@
     <t>i_zy</t>
   </si>
   <si>
-    <t>Nose</t>
-  </si>
-  <si>
-    <t>Cabin</t>
-  </si>
-  <si>
-    <t>Engine Fairings</t>
-  </si>
-  <si>
-    <t>Left Tailboom</t>
-  </si>
-  <si>
-    <t>Right Tailboom</t>
-  </si>
-  <si>
-    <t>Horizontal Tailplane</t>
-  </si>
-  <si>
-    <t>Left Vertical Tail</t>
-  </si>
-  <si>
-    <t>Right Vertical Tailplane</t>
-  </si>
-  <si>
     <t>Fuel Tanks</t>
   </si>
   <si>
-    <t>Engines, Transmission</t>
-  </si>
-  <si>
     <t>Elec, Hyd</t>
   </si>
   <si>
@@ -110,43 +83,52 @@
     <t>Battery</t>
   </si>
   <si>
-    <t>Pilots (and worn equipment)</t>
-  </si>
-  <si>
     <t>Rear pax</t>
   </si>
   <si>
-    <t>Crew radio</t>
-  </si>
-  <si>
     <t>Dashboard</t>
   </si>
   <si>
-    <t>Air data computers</t>
-  </si>
-  <si>
-    <t>Air Conditioning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Radio altimeter </t>
-  </si>
-  <si>
     <t xml:space="preserve">HTAWS </t>
   </si>
   <si>
     <t>FLIR 111</t>
   </si>
   <si>
-    <t>Wirestrike system</t>
-  </si>
-  <si>
     <t xml:space="preserve">Spotlight </t>
   </si>
   <si>
-    <t>Systems behind pilot (can be split up after intial granular cg)</t>
-  </si>
-  <si>
     <t>Floor</t>
+  </si>
+  <si>
+    <t>Structure</t>
+  </si>
+  <si>
+    <t>Cockpit</t>
+  </si>
+  <si>
+    <t>Avionics Bay</t>
+  </si>
+  <si>
+    <t>Environmental Control System</t>
+  </si>
+  <si>
+    <t>Data Cabling</t>
+  </si>
+  <si>
+    <t>Antennae pitot etc.</t>
+  </si>
+  <si>
+    <t>Control Systems</t>
+  </si>
+  <si>
+    <t>Transmission</t>
+  </si>
+  <si>
+    <t>Engines</t>
+  </si>
+  <si>
+    <t>Landing Gear</t>
   </si>
 </sst>
 </file>
@@ -464,10 +446,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -507,19 +489,19 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B2">
-        <v>8.3391999999999999</v>
+        <v>195.61080000000001</v>
       </c>
       <c r="C2">
-        <v>0.70799999999999996</v>
+        <v>3.7890000000000001</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0.93600000000000005</v>
+        <v>1.5309999999999999</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -542,19 +524,19 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3">
-        <v>116.16</v>
+        <v>761.1</v>
       </c>
       <c r="C3">
-        <v>3.9209999999999998</v>
+        <v>3.4</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1.351</v>
+        <v>0.58499999999999996</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -577,13 +559,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B4">
-        <v>30.540800000000001</v>
+        <v>306</v>
       </c>
       <c r="C4">
-        <v>4.9050000000000002</v>
+        <v>4.5</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -612,19 +594,19 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B5">
-        <v>6.03</v>
+        <v>188.8</v>
       </c>
       <c r="C5">
-        <v>8.5280000000000005</v>
+        <v>3.3</v>
       </c>
       <c r="D5">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>2.1259999999999999</v>
+        <v>2.5129999999999999</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -647,19 +629,19 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6">
-        <v>6.03</v>
+        <v>24.1</v>
       </c>
       <c r="C6">
-        <v>8.5280000000000005</v>
+        <v>3.8</v>
       </c>
       <c r="D6">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>2.1259999999999999</v>
+        <v>1.351</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -682,19 +664,19 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B7">
-        <v>18.12</v>
+        <v>462.15</v>
       </c>
       <c r="C7">
-        <v>10.077</v>
+        <v>3.5</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>2.1539999999999999</v>
+        <v>1.351</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -717,19 +699,19 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B8">
-        <v>6.37</v>
+        <v>19</v>
       </c>
       <c r="C8">
-        <v>10.099</v>
+        <v>2.5</v>
       </c>
       <c r="D8">
-        <v>-1.5760000000000001</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>2.1339999999999999</v>
+        <v>2</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -752,19 +734,19 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B9">
-        <v>6.37</v>
+        <v>286.76799999999997</v>
       </c>
       <c r="C9">
-        <v>10.099</v>
+        <v>0.875</v>
       </c>
       <c r="D9">
-        <v>1.5760000000000001</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>2.1339999999999999</v>
+        <v>1</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -787,13 +769,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B10">
-        <v>673</v>
+        <v>16.309999999999999</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>2.0190000000000001</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -822,19 +804,19 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B11">
-        <v>494.8</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="C11">
-        <v>4.8</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>2.5129999999999999</v>
+        <v>0.65</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -857,19 +839,20 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B12">
-        <v>24.1</v>
+        <f>90*4</f>
+        <v>360</v>
       </c>
       <c r="C12">
-        <v>3.9209999999999998</v>
+        <v>4</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>1.351</v>
+        <v>0</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -892,19 +875,19 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B13">
-        <v>462.15</v>
+        <v>53.87</v>
       </c>
       <c r="C13">
-        <v>3.9209999999999998</v>
+        <v>3.1619999999999999</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <v>1.351</v>
+        <v>0.6</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -927,19 +910,19 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B14">
-        <v>19</v>
+        <v>5.25</v>
       </c>
       <c r="C14">
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -965,17 +948,16 @@
         <v>24</v>
       </c>
       <c r="B15">
-        <f>2*(90+2+0.404)</f>
-        <v>184.80799999999999</v>
+        <v>50</v>
       </c>
       <c r="C15">
-        <v>1.9</v>
+        <v>5</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15">
-        <v>3</v>
+        <v>2.5129999999999999</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -998,20 +980,19 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B16">
-        <f>90*4</f>
-        <v>360</v>
+        <v>20</v>
       </c>
       <c r="C16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -1034,10 +1015,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B17">
-        <v>1.1000000000000001</v>
+        <v>31</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -1046,7 +1027,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1069,13 +1050,13 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B18">
-        <v>20.260000000000002</v>
+        <v>1.25</v>
       </c>
       <c r="C18">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -1104,19 +1085,19 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B19">
-        <v>1.71</v>
+        <v>20</v>
       </c>
       <c r="C19">
-        <v>0.70799999999999996</v>
+        <v>1.5</v>
       </c>
       <c r="D19">
         <v>0</v>
       </c>
       <c r="E19">
-        <v>0.93600000000000005</v>
+        <v>1</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1139,19 +1120,19 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B20">
         <v>50</v>
       </c>
       <c r="C20">
-        <v>5</v>
+        <v>2.02</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
       <c r="E20">
-        <v>2.5129999999999999</v>
+        <v>2.1</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -1177,16 +1158,16 @@
         <v>30</v>
       </c>
       <c r="B21">
-        <v>1.4</v>
+        <v>72</v>
       </c>
       <c r="C21">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1204,216 +1185,6 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>31</v>
-      </c>
-      <c r="B22">
-        <v>5.25</v>
-      </c>
-      <c r="C22">
-        <v>0.70799999999999996</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
-        <v>0.93600000000000005</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22">
-        <v>0</v>
-      </c>
-      <c r="H22">
-        <v>0</v>
-      </c>
-      <c r="I22">
-        <v>0</v>
-      </c>
-      <c r="J22">
-        <v>0</v>
-      </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>32</v>
-      </c>
-      <c r="B23">
-        <v>20</v>
-      </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23">
-        <v>0.6</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
-      <c r="I23">
-        <v>0</v>
-      </c>
-      <c r="J23">
-        <v>0</v>
-      </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24">
-        <v>7</v>
-      </c>
-      <c r="C24">
-        <v>2</v>
-      </c>
-      <c r="D24">
-        <v>0</v>
-      </c>
-      <c r="E24">
-        <v>1.8</v>
-      </c>
-      <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24">
-        <v>0</v>
-      </c>
-      <c r="H24">
-        <v>0</v>
-      </c>
-      <c r="I24">
-        <v>0</v>
-      </c>
-      <c r="J24">
-        <v>0</v>
-      </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>34</v>
-      </c>
-      <c r="B25">
-        <v>31</v>
-      </c>
-      <c r="C25">
-        <v>2</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25">
-        <v>0.6</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-      <c r="G25">
-        <v>0</v>
-      </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-      <c r="I25">
-        <v>0</v>
-      </c>
-      <c r="J25">
-        <v>0</v>
-      </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26">
-        <v>30</v>
-      </c>
-      <c r="C26">
-        <v>2.5299999999999998</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>1.8</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="H26">
-        <v>0</v>
-      </c>
-      <c r="I26">
-        <v>0</v>
-      </c>
-      <c r="J26">
-        <v>0</v>
-      </c>
-      <c r="K26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27">
-        <v>53.87</v>
-      </c>
-      <c r="C27">
-        <v>3.1619999999999999</v>
-      </c>
-      <c r="D27">
-        <v>0</v>
-      </c>
-      <c r="E27">
-        <v>0.6</v>
-      </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>0</v>
-      </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
-      <c r="J27">
-        <v>0</v>
-      </c>
-      <c r="K27">
         <v>0</v>
       </c>
     </row>

</xml_diff>